<commit_message>
facturas de septiembre, acceso tax free, imagenes_relacion y Para hacer
Archivos sueltos que no son de un cambio de código puntual:
- Administración/: facturas y nota de crédito al 2026-09-03
- Tax free/Acceso tax free.xlsx: actualización
- imagenes_relacion.csv: actualización
- Para hacer.docx

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xz2gnKMLBf3ZA2gmqt9jDF
</commit_message>
<xml_diff>
--- a/Tax free/Acceso tax free.xlsx
+++ b/Tax free/Acceso tax free.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Local</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Lucero.1066</t>
+  </si>
+  <si>
+    <t>ahora que es joyería no tiene tax free</t>
   </si>
 </sst>
 </file>
@@ -474,13 +477,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.453125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="16.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -491,7 +494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -502,7 +505,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -513,7 +516,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -524,7 +527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -535,7 +538,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
@@ -546,7 +549,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
@@ -556,8 +559,11 @@
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
     </row>
   </sheetData>

</xml_diff>